<commit_message>
BOM: replace CAN transceiver line with U6 and MCP2562FD-E/SN
Populate Microchip ordering data and notes (VDD/VIO supplies vs TJA1051T/3);
datasheet reference DS20005284.

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/esp32io-v1.01_BOM_PCBWay.xlsx
+++ b/esp32io-v1.01_BOM_PCBWay.xlsx
@@ -955,8 +955,6 @@
       <c r="C18" t="n">
         <v>1</v>
       </c>
-      <c r="D18" t="inlineStr"/>
-      <c r="E18" t="inlineStr"/>
       <c r="F18" t="inlineStr">
         <is>
           <t>ESP32-Module</t>
@@ -1113,17 +1111,25 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>U5</t>
+          <t>U6</t>
         </is>
       </c>
       <c r="C22" t="n">
         <v>1</v>
       </c>
-      <c r="D22" t="inlineStr"/>
-      <c r="E22" t="inlineStr"/>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Microchip Technology</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>MCP2562FD-E/SN</t>
+        </is>
+      </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>TJA1051T-3</t>
+          <t>IC HS CAN FD transceiver with VIO, standby, 8-SOIC extended temp (-40 to +125 C)</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1138,7 +1144,7 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>Mouser / schematic: 726-IFX1050GVIOXUMA1 No match in saved cart — fill Manufacturer / Mfg Part # manually.</t>
+          <t>Replaces obsolete IFX1050GVIOXUMA1 / TJA1051T-3 line item. MCP2562FD: VDD (pin 3)=4.5–5.5 V for transceiver; VIO (pin 5)=MCU I/O rail (typically 3.3 V). Not a single-supply 3.3 V drop-in for TJA1051T/3 — confirm schematic nets (5 V to VDD, 3.3 V to VIO) and pinout vs original IC before assembly. Datasheet: Microchip DS20005284.</t>
         </is>
       </c>
     </row>
@@ -1369,8 +1375,6 @@
       <c r="C28" t="n">
         <v>1</v>
       </c>
-      <c r="D28" t="inlineStr"/>
-      <c r="E28" t="inlineStr"/>
       <c r="F28" t="inlineStr">
         <is>
           <t>LEFT-EXT</t>
@@ -1404,8 +1408,6 @@
       <c r="C29" t="n">
         <v>1</v>
       </c>
-      <c r="D29" t="inlineStr"/>
-      <c r="E29" t="inlineStr"/>
       <c r="F29" t="inlineStr">
         <is>
           <t>RIGHT-EXT</t>

</xml_diff>

<commit_message>
BOM: restore U5 designator on CAN transceiver row (U6 is a different ref)
Keep MCP2562FD-E/SN substitution; only the refdes was wrong.

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/esp32io-v1.01_BOM_PCBWay.xlsx
+++ b/esp32io-v1.01_BOM_PCBWay.xlsx
@@ -1111,7 +1111,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>U6</t>
+          <t>U5</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -1144,7 +1144,7 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>Replaces obsolete IFX1050GVIOXUMA1 / TJA1051T-3 line item. MCP2562FD: VDD (pin 3)=4.5–5.5 V for transceiver; VIO (pin 5)=MCU I/O rail (typically 3.3 V). Not a single-supply 3.3 V drop-in for TJA1051T/3 — confirm schematic nets (5 V to VDD, 3.3 V to VIO) and pinout vs original IC before assembly. Datasheet: Microchip DS20005284.</t>
+          <t>Replaces obsolete IFX1050GVIOXUMA1 / CAN transceiver (designator U5 per KiCad export). MCP2562FD: VDD (pin 3)=4.5–5.5 V for transceiver; VIO (pin 5)=MCU I/O rail (typically 3.3 V). Not a single-supply 3.3 V drop-in for TJA1051T/3 — confirm schematic nets (5 V to VDD, 3.3 V to VIO) and pinout vs original IC before assembly. Datasheet: Microchip DS20005284.</t>
         </is>
       </c>
     </row>

</xml_diff>